<commit_message>
Correcciones en las mediciones
</commit_message>
<xml_diff>
--- a/Codigos de simulación/Datos Experimentales/2025-04-02 Mediciones del perfil.xlsx
+++ b/Codigos de simulación/Datos Experimentales/2025-04-02 Mediciones del perfil.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G67"/>
+  <dimension ref="A1:I67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,1536 +451,1942 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>y</t>
+          <t>w1</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>w2</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>w3</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>sigma</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>w</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>40</v>
+        <v>-40</v>
       </c>
       <c r="C2" t="n">
-        <v>39.9</v>
+        <v>-39.9</v>
       </c>
       <c r="D2" t="n">
-        <v>40.2</v>
+        <v>-40.2</v>
       </c>
       <c r="E2" t="n">
-        <v>40.03333333333334</v>
+        <v>-22.5</v>
       </c>
       <c r="F2" t="n">
+        <v>-22.4</v>
+      </c>
+      <c r="G2" t="n">
+        <v>-22.7</v>
+      </c>
+      <c r="H2" t="n">
+        <v>-22.53333333333333</v>
+      </c>
+      <c r="I2" t="n">
         <v>0.08819171036882094</v>
-      </c>
-      <c r="G2" t="n">
-        <v>22.53333333333334</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>64</v>
+        <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>39.85</v>
+        <v>-39.85</v>
       </c>
       <c r="C3" t="n">
-        <v>39.95</v>
+        <v>-39.95</v>
       </c>
       <c r="D3" t="n">
-        <v>39.85</v>
+        <v>-39.85</v>
       </c>
       <c r="E3" t="n">
-        <v>39.88333333333333</v>
+        <v>-22.35</v>
       </c>
       <c r="F3" t="n">
+        <v>-22.45</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-22.35</v>
+      </c>
+      <c r="H3" t="n">
+        <v>-22.38333333333334</v>
+      </c>
+      <c r="I3" t="n">
         <v>0.03333333333333381</v>
-      </c>
-      <c r="G3" t="n">
-        <v>22.38333333333333</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>63</v>
+        <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>40.27</v>
+        <v>-40.27</v>
       </c>
       <c r="C4" t="n">
-        <v>40.47</v>
+        <v>-40.47</v>
       </c>
       <c r="D4" t="n">
-        <v>40.37</v>
+        <v>-40.37</v>
       </c>
       <c r="E4" t="n">
-        <v>40.37</v>
+        <v>-22.77</v>
       </c>
       <c r="F4" t="n">
-        <v>0.05773502691896136</v>
+        <v>-22.97</v>
       </c>
       <c r="G4" t="n">
-        <v>22.87</v>
+        <v>-22.87</v>
+      </c>
+      <c r="H4" t="n">
+        <v>-22.87</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.05773502691896135</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>62</v>
+        <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>38.4</v>
+        <v>-38.4</v>
       </c>
       <c r="C5" t="n">
-        <v>38.5</v>
+        <v>-38.5</v>
       </c>
       <c r="D5" t="n">
-        <v>38.5</v>
+        <v>-38.5</v>
       </c>
       <c r="E5" t="n">
-        <v>38.46666666666667</v>
+        <v>-20.9</v>
       </c>
       <c r="F5" t="n">
+        <v>-21</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-21</v>
+      </c>
+      <c r="H5" t="n">
+        <v>-20.96666666666667</v>
+      </c>
+      <c r="I5" t="n">
         <v>0.03333333333333381</v>
-      </c>
-      <c r="G5" t="n">
-        <v>20.96666666666667</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>61</v>
+        <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>38.4</v>
+        <v>-38.4</v>
       </c>
       <c r="C6" t="n">
-        <v>38.4</v>
+        <v>-38.4</v>
       </c>
       <c r="D6" t="n">
-        <v>38.5</v>
+        <v>-38.5</v>
       </c>
       <c r="E6" t="n">
-        <v>38.43333333333333</v>
+        <v>-20.9</v>
       </c>
       <c r="F6" t="n">
+        <v>-20.9</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-21</v>
+      </c>
+      <c r="H6" t="n">
+        <v>-20.93333333333333</v>
+      </c>
+      <c r="I6" t="n">
         <v>0.03333333333333381</v>
-      </c>
-      <c r="G6" t="n">
-        <v>20.93333333333333</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>60</v>
+        <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>37.3</v>
+        <v>-37.3</v>
       </c>
       <c r="C7" t="n">
-        <v>37.6</v>
+        <v>-37.6</v>
       </c>
       <c r="D7" t="n">
-        <v>37.3</v>
+        <v>-37.3</v>
       </c>
       <c r="E7" t="n">
-        <v>37.4</v>
+        <v>-19.8</v>
       </c>
       <c r="F7" t="n">
+        <v>-20.1</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-19.8</v>
+      </c>
+      <c r="H7" t="n">
+        <v>-19.9</v>
+      </c>
+      <c r="I7" t="n">
         <v>0.1000000000000014</v>
-      </c>
-      <c r="G7" t="n">
-        <v>19.9</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>59</v>
+        <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>36.5</v>
+        <v>-36.5</v>
       </c>
       <c r="C8" t="n">
-        <v>36.5</v>
+        <v>-36.5</v>
       </c>
       <c r="D8" t="n">
-        <v>36.6</v>
+        <v>-36.6</v>
       </c>
       <c r="E8" t="n">
-        <v>36.53333333333333</v>
+        <v>-19</v>
       </c>
       <c r="F8" t="n">
+        <v>-19</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-19.1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>-19.03333333333333</v>
+      </c>
+      <c r="I8" t="n">
         <v>0.03333333333333381</v>
-      </c>
-      <c r="G8" t="n">
-        <v>19.03333333333333</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>58</v>
+        <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>35.8</v>
+        <v>-35.8</v>
       </c>
       <c r="C9" t="n">
-        <v>35.6</v>
+        <v>-35.6</v>
       </c>
       <c r="D9" t="n">
-        <v>35.7</v>
+        <v>-35.7</v>
       </c>
       <c r="E9" t="n">
-        <v>35.7</v>
+        <v>-18.3</v>
       </c>
       <c r="F9" t="n">
-        <v>0.05773502691896136</v>
+        <v>-18.1</v>
       </c>
       <c r="G9" t="n">
-        <v>18.2</v>
+        <v>-18.2</v>
+      </c>
+      <c r="H9" t="n">
+        <v>-18.2</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.05773502691896135</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>57</v>
+        <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>35.1</v>
+        <v>-35.1</v>
       </c>
       <c r="C10" t="n">
-        <v>34.9</v>
+        <v>-34.9</v>
       </c>
       <c r="D10" t="n">
-        <v>35.2</v>
+        <v>-35.2</v>
       </c>
       <c r="E10" t="n">
-        <v>35.06666666666667</v>
+        <v>-17.6</v>
       </c>
       <c r="F10" t="n">
+        <v>-17.4</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-17.7</v>
+      </c>
+      <c r="H10" t="n">
+        <v>-17.56666666666667</v>
+      </c>
+      <c r="I10" t="n">
         <v>0.08819171036882094</v>
-      </c>
-      <c r="G10" t="n">
-        <v>17.56666666666667</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>56</v>
+        <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>34.8</v>
+        <v>-34.8</v>
       </c>
       <c r="C11" t="n">
-        <v>35</v>
+        <v>-35</v>
       </c>
       <c r="D11" t="n">
-        <v>35.2</v>
+        <v>-35.2</v>
       </c>
       <c r="E11" t="n">
-        <v>35</v>
+        <v>-17.3</v>
       </c>
       <c r="F11" t="n">
+        <v>-17.5</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-17.7</v>
+      </c>
+      <c r="H11" t="n">
+        <v>-17.5</v>
+      </c>
+      <c r="I11" t="n">
         <v>0.1154700538379268</v>
-      </c>
-      <c r="G11" t="n">
-        <v>17.5</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>34.6</v>
+        <v>-34.6</v>
       </c>
       <c r="C12" t="n">
-        <v>34.4</v>
+        <v>-34.4</v>
       </c>
       <c r="D12" t="n">
-        <v>34.4</v>
+        <v>-34.4</v>
       </c>
       <c r="E12" t="n">
-        <v>34.46666666666667</v>
+        <v>-17.1</v>
       </c>
       <c r="F12" t="n">
+        <v>-16.9</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-16.9</v>
+      </c>
+      <c r="H12" t="n">
+        <v>-16.96666666666667</v>
+      </c>
+      <c r="I12" t="n">
         <v>0.06666666666666762</v>
-      </c>
-      <c r="G12" t="n">
-        <v>16.96666666666667</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>54</v>
+        <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>33.5</v>
+        <v>-33.5</v>
       </c>
       <c r="C13" t="n">
-        <v>33.8</v>
+        <v>-33.8</v>
       </c>
       <c r="D13" t="n">
-        <v>33.7</v>
+        <v>-33.7</v>
       </c>
       <c r="E13" t="n">
-        <v>33.66666666666666</v>
+        <v>-16</v>
       </c>
       <c r="F13" t="n">
+        <v>-16.3</v>
+      </c>
+      <c r="G13" t="n">
+        <v>-16.2</v>
+      </c>
+      <c r="H13" t="n">
+        <v>-16.16666666666667</v>
+      </c>
+      <c r="I13" t="n">
         <v>0.08819171036881916</v>
-      </c>
-      <c r="G13" t="n">
-        <v>16.16666666666666</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>53</v>
+        <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>32.5</v>
+        <v>-32.5</v>
       </c>
       <c r="C14" t="n">
-        <v>32.8</v>
+        <v>-32.8</v>
       </c>
       <c r="D14" t="n">
-        <v>32.6</v>
+        <v>-32.6</v>
       </c>
       <c r="E14" t="n">
-        <v>32.63333333333333</v>
+        <v>-15</v>
       </c>
       <c r="F14" t="n">
+        <v>-15.3</v>
+      </c>
+      <c r="G14" t="n">
+        <v>-15.1</v>
+      </c>
+      <c r="H14" t="n">
+        <v>-15.13333333333333</v>
+      </c>
+      <c r="I14" t="n">
         <v>0.08819171036881872</v>
-      </c>
-      <c r="G14" t="n">
-        <v>15.13333333333333</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>52</v>
+        <v>13</v>
       </c>
       <c r="B15" t="n">
-        <v>32.5</v>
+        <v>-32.5</v>
       </c>
       <c r="C15" t="n">
-        <v>33.2</v>
+        <v>-33.2</v>
       </c>
       <c r="D15" t="n">
-        <v>32.6</v>
+        <v>-32.6</v>
       </c>
       <c r="E15" t="n">
-        <v>32.76666666666667</v>
+        <v>-15</v>
       </c>
       <c r="F15" t="n">
+        <v>-15.7</v>
+      </c>
+      <c r="G15" t="n">
+        <v>-15.1</v>
+      </c>
+      <c r="H15" t="n">
+        <v>-15.26666666666667</v>
+      </c>
+      <c r="I15" t="n">
         <v>0.2185812841434008</v>
-      </c>
-      <c r="G15" t="n">
-        <v>15.26666666666667</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>51</v>
+        <v>14</v>
       </c>
       <c r="B16" t="n">
-        <v>32.2</v>
+        <v>-32.2</v>
       </c>
       <c r="C16" t="n">
-        <v>32.1</v>
+        <v>-32.1</v>
       </c>
       <c r="D16" t="n">
-        <v>32.2</v>
+        <v>-32.2</v>
       </c>
       <c r="E16" t="n">
-        <v>32.16666666666667</v>
+        <v>-14.7</v>
       </c>
       <c r="F16" t="n">
+        <v>-14.6</v>
+      </c>
+      <c r="G16" t="n">
+        <v>-14.7</v>
+      </c>
+      <c r="H16" t="n">
+        <v>-14.66666666666667</v>
+      </c>
+      <c r="I16" t="n">
         <v>0.03333333333333381</v>
-      </c>
-      <c r="G16" t="n">
-        <v>14.66666666666667</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="B17" t="n">
-        <v>31.8</v>
+        <v>-31.8</v>
       </c>
       <c r="C17" t="n">
-        <v>31.6</v>
+        <v>-31.6</v>
       </c>
       <c r="D17" t="n">
-        <v>31.8</v>
+        <v>-31.8</v>
       </c>
       <c r="E17" t="n">
-        <v>31.73333333333333</v>
+        <v>-14.3</v>
       </c>
       <c r="F17" t="n">
+        <v>-14.1</v>
+      </c>
+      <c r="G17" t="n">
+        <v>-14.3</v>
+      </c>
+      <c r="H17" t="n">
+        <v>-14.23333333333333</v>
+      </c>
+      <c r="I17" t="n">
         <v>0.06666666666666643</v>
-      </c>
-      <c r="G17" t="n">
-        <v>14.23333333333333</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>49</v>
+        <v>16</v>
       </c>
       <c r="B18" t="n">
-        <v>31.4</v>
+        <v>-31.4</v>
       </c>
       <c r="C18" t="n">
-        <v>31.4</v>
+        <v>-31.4</v>
       </c>
       <c r="D18" t="n">
-        <v>31.5</v>
+        <v>-31.5</v>
       </c>
       <c r="E18" t="n">
-        <v>31.43333333333333</v>
+        <v>-13.9</v>
       </c>
       <c r="F18" t="n">
+        <v>-13.9</v>
+      </c>
+      <c r="G18" t="n">
+        <v>-14</v>
+      </c>
+      <c r="H18" t="n">
+        <v>-13.93333333333333</v>
+      </c>
+      <c r="I18" t="n">
         <v>0.03333333333333381</v>
-      </c>
-      <c r="G18" t="n">
-        <v>13.93333333333333</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>48</v>
+        <v>17</v>
       </c>
       <c r="B19" t="n">
-        <v>31.1</v>
+        <v>-31.1</v>
       </c>
       <c r="C19" t="n">
-        <v>31.2</v>
+        <v>-31.2</v>
       </c>
       <c r="D19" t="n">
-        <v>30.9</v>
+        <v>-30.9</v>
       </c>
       <c r="E19" t="n">
-        <v>31.06666666666666</v>
+        <v>-13.6</v>
       </c>
       <c r="F19" t="n">
+        <v>-13.7</v>
+      </c>
+      <c r="G19" t="n">
+        <v>-13.4</v>
+      </c>
+      <c r="H19" t="n">
+        <v>-13.56666666666667</v>
+      </c>
+      <c r="I19" t="n">
         <v>0.08819171036882006</v>
-      </c>
-      <c r="G19" t="n">
-        <v>13.56666666666666</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>47</v>
+        <v>18</v>
       </c>
       <c r="B20" t="n">
-        <v>30.6</v>
+        <v>-30.6</v>
       </c>
       <c r="C20" t="n">
-        <v>30.5</v>
+        <v>-30.5</v>
       </c>
       <c r="D20" t="n">
-        <v>30.7</v>
+        <v>-30.7</v>
       </c>
       <c r="E20" t="n">
-        <v>30.6</v>
+        <v>-13.1</v>
       </c>
       <c r="F20" t="n">
+        <v>-13</v>
+      </c>
+      <c r="G20" t="n">
+        <v>-13.2</v>
+      </c>
+      <c r="H20" t="n">
+        <v>-13.1</v>
+      </c>
+      <c r="I20" t="n">
         <v>0.05773502691896237</v>
-      </c>
-      <c r="G20" t="n">
-        <v>13.1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="B21" t="n">
-        <v>30.5</v>
+        <v>-30.5</v>
       </c>
       <c r="C21" t="n">
-        <v>29.9</v>
+        <v>-29.9</v>
       </c>
       <c r="D21" t="n">
-        <v>30.2</v>
+        <v>-30.2</v>
       </c>
       <c r="E21" t="n">
-        <v>30.2</v>
+        <v>-13</v>
       </c>
       <c r="F21" t="n">
+        <v>-12.4</v>
+      </c>
+      <c r="G21" t="n">
+        <v>-12.7</v>
+      </c>
+      <c r="H21" t="n">
+        <v>-12.7</v>
+      </c>
+      <c r="I21" t="n">
         <v>0.1732050807568881</v>
-      </c>
-      <c r="G21" t="n">
-        <v>12.7</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="B22" t="n">
-        <v>29.9</v>
+        <v>-29.9</v>
       </c>
       <c r="C22" t="n">
-        <v>30</v>
+        <v>-30</v>
       </c>
       <c r="D22" t="n">
-        <v>30.1</v>
+        <v>-30.1</v>
       </c>
       <c r="E22" t="n">
-        <v>30</v>
+        <v>-12.4</v>
       </c>
       <c r="F22" t="n">
+        <v>-12.5</v>
+      </c>
+      <c r="G22" t="n">
+        <v>-12.6</v>
+      </c>
+      <c r="H22" t="n">
+        <v>-12.5</v>
+      </c>
+      <c r="I22" t="n">
         <v>0.0577350269189634</v>
-      </c>
-      <c r="G22" t="n">
-        <v>12.5</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="B23" t="n">
-        <v>29.9</v>
+        <v>-29.9</v>
       </c>
       <c r="C23" t="n">
-        <v>30</v>
+        <v>-30</v>
       </c>
       <c r="D23" t="n">
-        <v>29.7</v>
+        <v>-29.7</v>
       </c>
       <c r="E23" t="n">
-        <v>29.86666666666666</v>
+        <v>-12.4</v>
       </c>
       <c r="F23" t="n">
+        <v>-12.5</v>
+      </c>
+      <c r="G23" t="n">
+        <v>-12.2</v>
+      </c>
+      <c r="H23" t="n">
+        <v>-12.36666666666667</v>
+      </c>
+      <c r="I23" t="n">
         <v>0.08819171036881983</v>
-      </c>
-      <c r="G23" t="n">
-        <v>12.36666666666666</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>43</v>
+        <v>22</v>
       </c>
       <c r="B24" t="n">
-        <v>29.1</v>
+        <v>-29.1</v>
       </c>
       <c r="C24" t="n">
-        <v>29.2</v>
+        <v>-29.2</v>
       </c>
       <c r="D24" t="n">
-        <v>29.3</v>
+        <v>-29.3</v>
       </c>
       <c r="E24" t="n">
-        <v>29.2</v>
+        <v>-11.6</v>
       </c>
       <c r="F24" t="n">
+        <v>-11.7</v>
+      </c>
+      <c r="G24" t="n">
+        <v>-11.8</v>
+      </c>
+      <c r="H24" t="n">
+        <v>-11.7</v>
+      </c>
+      <c r="I24" t="n">
         <v>0.05773502691896237</v>
-      </c>
-      <c r="G24" t="n">
-        <v>11.7</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="B25" t="n">
-        <v>28.7</v>
+        <v>-28.7</v>
       </c>
       <c r="C25" t="n">
-        <v>29.1</v>
+        <v>-29.1</v>
       </c>
       <c r="D25" t="n">
-        <v>29.2</v>
+        <v>-29.2</v>
       </c>
       <c r="E25" t="n">
-        <v>29</v>
+        <v>-11.2</v>
       </c>
       <c r="F25" t="n">
+        <v>-11.6</v>
+      </c>
+      <c r="G25" t="n">
+        <v>-11.7</v>
+      </c>
+      <c r="H25" t="n">
+        <v>-11.5</v>
+      </c>
+      <c r="I25" t="n">
         <v>0.1527525231651949</v>
-      </c>
-      <c r="G25" t="n">
-        <v>11.5</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>41</v>
+        <v>24</v>
       </c>
       <c r="B26" t="n">
-        <v>28.5</v>
+        <v>-28.5</v>
       </c>
       <c r="C26" t="n">
-        <v>28.8</v>
+        <v>-28.8</v>
       </c>
       <c r="D26" t="n">
-        <v>28.7</v>
+        <v>-28.7</v>
       </c>
       <c r="E26" t="n">
-        <v>28.66666666666667</v>
+        <v>-11</v>
       </c>
       <c r="F26" t="n">
-        <v>0.08819171036881981</v>
+        <v>-11.3</v>
       </c>
       <c r="G26" t="n">
-        <v>11.16666666666667</v>
+        <v>-11.2</v>
+      </c>
+      <c r="H26" t="n">
+        <v>-11.16666666666667</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0.08819171036881983</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="B27" t="n">
-        <v>28.3</v>
+        <v>-28.3</v>
       </c>
       <c r="C27" t="n">
-        <v>28.4</v>
+        <v>-28.4</v>
       </c>
       <c r="D27" t="n">
-        <v>28.3</v>
+        <v>-28.3</v>
       </c>
       <c r="E27" t="n">
-        <v>28.33333333333333</v>
+        <v>-10.8</v>
       </c>
       <c r="F27" t="n">
+        <v>-10.9</v>
+      </c>
+      <c r="G27" t="n">
+        <v>-10.8</v>
+      </c>
+      <c r="H27" t="n">
+        <v>-10.83333333333333</v>
+      </c>
+      <c r="I27" t="n">
         <v>0.03333333333333263</v>
-      </c>
-      <c r="G27" t="n">
-        <v>10.83333333333333</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="B28" t="n">
-        <v>28.4</v>
+        <v>-28.4</v>
       </c>
       <c r="C28" t="n">
-        <v>28.2</v>
+        <v>-28.2</v>
       </c>
       <c r="D28" t="n">
-        <v>27.6</v>
+        <v>-27.6</v>
       </c>
       <c r="E28" t="n">
-        <v>28.06666666666666</v>
+        <v>-10.9</v>
       </c>
       <c r="F28" t="n">
+        <v>-10.7</v>
+      </c>
+      <c r="G28" t="n">
+        <v>-10.1</v>
+      </c>
+      <c r="H28" t="n">
+        <v>-10.56666666666667</v>
+      </c>
+      <c r="I28" t="n">
         <v>0.2403700850309318</v>
-      </c>
-      <c r="G28" t="n">
-        <v>10.56666666666666</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="B29" t="n">
-        <v>27.9</v>
+        <v>-27.9</v>
       </c>
       <c r="C29" t="n">
-        <v>27.9</v>
+        <v>-27.9</v>
       </c>
       <c r="D29" t="n">
-        <v>28</v>
+        <v>-28</v>
       </c>
       <c r="E29" t="n">
-        <v>27.93333333333333</v>
+        <v>-10.4</v>
       </c>
       <c r="F29" t="n">
+        <v>-10.4</v>
+      </c>
+      <c r="G29" t="n">
+        <v>-10.5</v>
+      </c>
+      <c r="H29" t="n">
+        <v>-10.43333333333333</v>
+      </c>
+      <c r="I29" t="n">
         <v>0.03333333333333381</v>
-      </c>
-      <c r="G29" t="n">
-        <v>10.43333333333333</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="B30" t="n">
-        <v>27.8</v>
+        <v>-27.8</v>
       </c>
       <c r="C30" t="n">
-        <v>27.5</v>
+        <v>-27.5</v>
       </c>
       <c r="D30" t="n">
-        <v>28</v>
+        <v>-28</v>
       </c>
       <c r="E30" t="n">
-        <v>27.76666666666667</v>
+        <v>-10.3</v>
       </c>
       <c r="F30" t="n">
+        <v>-10</v>
+      </c>
+      <c r="G30" t="n">
+        <v>-10.5</v>
+      </c>
+      <c r="H30" t="n">
+        <v>-10.26666666666667</v>
+      </c>
+      <c r="I30" t="n">
         <v>0.1452966314513558</v>
-      </c>
-      <c r="G30" t="n">
-        <v>10.26666666666667</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B31" t="n">
-        <v>27.2</v>
+        <v>-27.2</v>
       </c>
       <c r="C31" t="n">
-        <v>27.4</v>
+        <v>-27.4</v>
       </c>
       <c r="D31" t="n">
-        <v>27.5</v>
+        <v>-27.5</v>
       </c>
       <c r="E31" t="n">
-        <v>27.36666666666666</v>
+        <v>-9.699999999999999</v>
       </c>
       <c r="F31" t="n">
+        <v>-9.899999999999999</v>
+      </c>
+      <c r="G31" t="n">
+        <v>-10</v>
+      </c>
+      <c r="H31" t="n">
+        <v>-9.866666666666665</v>
+      </c>
+      <c r="I31" t="n">
         <v>0.08819171036881983</v>
-      </c>
-      <c r="G31" t="n">
-        <v>9.866666666666664</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B32" t="n">
-        <v>26.6</v>
+        <v>-26.6</v>
       </c>
       <c r="C32" t="n">
-        <v>26.8</v>
+        <v>-26.8</v>
       </c>
       <c r="D32" t="n">
-        <v>26.7</v>
+        <v>-26.7</v>
       </c>
       <c r="E32" t="n">
-        <v>26.7</v>
+        <v>-9.100000000000001</v>
       </c>
       <c r="F32" t="n">
+        <v>-9.300000000000001</v>
+      </c>
+      <c r="G32" t="n">
+        <v>-9.199999999999999</v>
+      </c>
+      <c r="H32" t="n">
+        <v>-9.200000000000001</v>
+      </c>
+      <c r="I32" t="n">
         <v>0.05773502691896237</v>
-      </c>
-      <c r="G32" t="n">
-        <v>9.200000000000003</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B33" t="n">
-        <v>26.6</v>
+        <v>-26.6</v>
       </c>
       <c r="C33" t="n">
-        <v>26.5</v>
+        <v>-26.5</v>
       </c>
       <c r="D33" t="n">
-        <v>26.6</v>
+        <v>-26.6</v>
       </c>
       <c r="E33" t="n">
-        <v>26.56666666666667</v>
+        <v>-9.100000000000001</v>
       </c>
       <c r="F33" t="n">
+        <v>-9</v>
+      </c>
+      <c r="G33" t="n">
+        <v>-9.100000000000001</v>
+      </c>
+      <c r="H33" t="n">
+        <v>-9.066666666666668</v>
+      </c>
+      <c r="I33" t="n">
         <v>0.03333333333333381</v>
-      </c>
-      <c r="G33" t="n">
-        <v>9.066666666666666</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B34" t="n">
-        <v>26.5</v>
+        <v>-26.5</v>
       </c>
       <c r="C34" t="n">
-        <v>26.2</v>
+        <v>-26.2</v>
       </c>
       <c r="D34" t="n">
-        <v>26</v>
+        <v>-26</v>
       </c>
       <c r="E34" t="n">
-        <v>26.23333333333333</v>
+        <v>-9</v>
       </c>
       <c r="F34" t="n">
+        <v>-8.699999999999999</v>
+      </c>
+      <c r="G34" t="n">
+        <v>-8.5</v>
+      </c>
+      <c r="H34" t="n">
+        <v>-8.733333333333333</v>
+      </c>
+      <c r="I34" t="n">
         <v>0.1452966314513558</v>
-      </c>
-      <c r="G34" t="n">
-        <v>8.733333333333334</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B35" t="n">
-        <v>25.8</v>
+        <v>-25.8</v>
       </c>
       <c r="C35" t="n">
-        <v>25.8</v>
+        <v>-25.8</v>
       </c>
       <c r="D35" t="n">
-        <v>25.9</v>
+        <v>-25.9</v>
       </c>
       <c r="E35" t="n">
-        <v>25.83333333333333</v>
+        <v>-8.300000000000001</v>
       </c>
       <c r="F35" t="n">
+        <v>-8.300000000000001</v>
+      </c>
+      <c r="G35" t="n">
+        <v>-8.399999999999999</v>
+      </c>
+      <c r="H35" t="n">
+        <v>-8.333333333333334</v>
+      </c>
+      <c r="I35" t="n">
         <v>0.03333333333333263</v>
-      </c>
-      <c r="G35" t="n">
-        <v>8.333333333333332</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B36" t="n">
-        <v>25.5</v>
+        <v>-25.5</v>
       </c>
       <c r="C36" t="n">
-        <v>25.6</v>
+        <v>-25.6</v>
       </c>
       <c r="D36" t="n">
-        <v>25.6</v>
+        <v>-25.6</v>
       </c>
       <c r="E36" t="n">
-        <v>25.56666666666667</v>
+        <v>-8</v>
       </c>
       <c r="F36" t="n">
+        <v>-8.100000000000001</v>
+      </c>
+      <c r="G36" t="n">
+        <v>-8.100000000000001</v>
+      </c>
+      <c r="H36" t="n">
+        <v>-8.066666666666668</v>
+      </c>
+      <c r="I36" t="n">
         <v>0.03333333333333381</v>
-      </c>
-      <c r="G36" t="n">
-        <v>8.066666666666666</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="B37" t="n">
-        <v>25.3</v>
+        <v>-25.3</v>
       </c>
       <c r="C37" t="n">
-        <v>25.2</v>
+        <v>-25.2</v>
       </c>
       <c r="D37" t="n">
-        <v>25.4</v>
+        <v>-25.4</v>
       </c>
       <c r="E37" t="n">
-        <v>25.3</v>
+        <v>-7.800000000000001</v>
       </c>
       <c r="F37" t="n">
+        <v>-7.699999999999999</v>
+      </c>
+      <c r="G37" t="n">
+        <v>-7.899999999999999</v>
+      </c>
+      <c r="H37" t="n">
+        <v>-7.8</v>
+      </c>
+      <c r="I37" t="n">
         <v>0.05773502691896237</v>
-      </c>
-      <c r="G37" t="n">
-        <v>7.800000000000001</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="B38" t="n">
-        <v>25.5</v>
+        <v>-25.5</v>
       </c>
       <c r="C38" t="n">
-        <v>25.2</v>
+        <v>-25.2</v>
       </c>
       <c r="D38" t="n">
-        <v>25.1</v>
+        <v>-25.1</v>
       </c>
       <c r="E38" t="n">
-        <v>25.26666666666667</v>
+        <v>-8</v>
       </c>
       <c r="F38" t="n">
+        <v>-7.699999999999999</v>
+      </c>
+      <c r="G38" t="n">
+        <v>-7.600000000000001</v>
+      </c>
+      <c r="H38" t="n">
+        <v>-7.766666666666667</v>
+      </c>
+      <c r="I38" t="n">
         <v>0.1201850425154661</v>
-      </c>
-      <c r="G38" t="n">
-        <v>7.766666666666669</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="B39" t="n">
-        <v>24.8</v>
+        <v>-24.8</v>
       </c>
       <c r="C39" t="n">
-        <v>24.6</v>
+        <v>-24.6</v>
       </c>
       <c r="D39" t="n">
-        <v>24.5</v>
+        <v>-24.5</v>
       </c>
       <c r="E39" t="n">
-        <v>24.63333333333334</v>
+        <v>-7.300000000000001</v>
       </c>
       <c r="F39" t="n">
+        <v>-7.100000000000001</v>
+      </c>
+      <c r="G39" t="n">
+        <v>-7</v>
+      </c>
+      <c r="H39" t="n">
+        <v>-7.133333333333334</v>
+      </c>
+      <c r="I39" t="n">
         <v>0.08819171036881983</v>
-      </c>
-      <c r="G39" t="n">
-        <v>7.133333333333336</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="B40" t="n">
-        <v>24.2</v>
+        <v>-24.2</v>
       </c>
       <c r="C40" t="n">
-        <v>24.1</v>
+        <v>-24.1</v>
       </c>
       <c r="D40" t="n">
-        <v>24</v>
+        <v>-24</v>
       </c>
       <c r="E40" t="n">
-        <v>24.1</v>
+        <v>-6.699999999999999</v>
       </c>
       <c r="F40" t="n">
+        <v>-6.600000000000001</v>
+      </c>
+      <c r="G40" t="n">
+        <v>-6.5</v>
+      </c>
+      <c r="H40" t="n">
+        <v>-6.600000000000001</v>
+      </c>
+      <c r="I40" t="n">
         <v>0.05773502691896237</v>
-      </c>
-      <c r="G40" t="n">
-        <v>6.599999999999998</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="B41" t="n">
-        <v>24.2</v>
+        <v>-24.2</v>
       </c>
       <c r="C41" t="n">
-        <v>23.9</v>
+        <v>-23.9</v>
       </c>
       <c r="D41" t="n">
-        <v>23.8</v>
+        <v>-23.8</v>
       </c>
       <c r="E41" t="n">
-        <v>23.96666666666667</v>
+        <v>-6.699999999999999</v>
       </c>
       <c r="F41" t="n">
+        <v>-6.399999999999999</v>
+      </c>
+      <c r="G41" t="n">
+        <v>-6.300000000000001</v>
+      </c>
+      <c r="H41" t="n">
+        <v>-6.466666666666666</v>
+      </c>
+      <c r="I41" t="n">
         <v>0.1201850425154661</v>
-      </c>
-      <c r="G41" t="n">
-        <v>6.466666666666665</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="B42" t="n">
-        <v>23.7</v>
+        <v>-23.7</v>
       </c>
       <c r="C42" t="n">
-        <v>23.8</v>
+        <v>-23.8</v>
       </c>
       <c r="D42" t="n">
-        <v>23.8</v>
+        <v>-23.8</v>
       </c>
       <c r="E42" t="n">
-        <v>23.76666666666667</v>
+        <v>-6.199999999999999</v>
       </c>
       <c r="F42" t="n">
+        <v>-6.300000000000001</v>
+      </c>
+      <c r="G42" t="n">
+        <v>-6.300000000000001</v>
+      </c>
+      <c r="H42" t="n">
+        <v>-6.266666666666667</v>
+      </c>
+      <c r="I42" t="n">
         <v>0.03333333333333381</v>
-      </c>
-      <c r="G42" t="n">
-        <v>6.266666666666666</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="B43" t="n">
-        <v>23.5</v>
+        <v>-23.5</v>
       </c>
       <c r="C43" t="n">
-        <v>23.5</v>
+        <v>-23.5</v>
       </c>
       <c r="D43" t="n">
-        <v>23.6</v>
+        <v>-23.6</v>
       </c>
       <c r="E43" t="n">
-        <v>23.53333333333333</v>
+        <v>-6</v>
       </c>
       <c r="F43" t="n">
+        <v>-6</v>
+      </c>
+      <c r="G43" t="n">
+        <v>-6.100000000000001</v>
+      </c>
+      <c r="H43" t="n">
+        <v>-6.033333333333334</v>
+      </c>
+      <c r="I43" t="n">
         <v>0.03333333333333381</v>
-      </c>
-      <c r="G43" t="n">
-        <v>6.033333333333331</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="B44" t="n">
-        <v>23.5</v>
+        <v>-23.5</v>
       </c>
       <c r="C44" t="n">
-        <v>23.4</v>
+        <v>-23.4</v>
       </c>
       <c r="D44" t="n">
-        <v>23.7</v>
+        <v>-23.7</v>
       </c>
       <c r="E44" t="n">
-        <v>23.53333333333333</v>
+        <v>-6</v>
       </c>
       <c r="F44" t="n">
-        <v>0.08819171036881981</v>
+        <v>-5.899999999999999</v>
       </c>
       <c r="G44" t="n">
-        <v>6.033333333333331</v>
+        <v>-6.199999999999999</v>
+      </c>
+      <c r="H44" t="n">
+        <v>-6.033333333333332</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0.08819171036881983</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>22</v>
+        <v>43</v>
       </c>
       <c r="B45" t="n">
-        <v>23</v>
+        <v>-23</v>
       </c>
       <c r="C45" t="n">
-        <v>23.5</v>
+        <v>-23.5</v>
       </c>
       <c r="D45" t="n">
-        <v>23.3</v>
+        <v>-23.3</v>
       </c>
       <c r="E45" t="n">
-        <v>23.26666666666667</v>
+        <v>-5.5</v>
       </c>
       <c r="F45" t="n">
+        <v>-6</v>
+      </c>
+      <c r="G45" t="n">
+        <v>-5.800000000000001</v>
+      </c>
+      <c r="H45" t="n">
+        <v>-5.766666666666667</v>
+      </c>
+      <c r="I45" t="n">
         <v>0.1452966314513558</v>
-      </c>
-      <c r="G45" t="n">
-        <v>5.766666666666666</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="B46" t="n">
-        <v>22.7</v>
+        <v>-22.7</v>
       </c>
       <c r="C46" t="n">
-        <v>22.4</v>
+        <v>-22.4</v>
       </c>
       <c r="D46" t="n">
-        <v>22.6</v>
+        <v>-22.6</v>
       </c>
       <c r="E46" t="n">
-        <v>22.56666666666666</v>
+        <v>-5.199999999999999</v>
       </c>
       <c r="F46" t="n">
+        <v>-4.899999999999999</v>
+      </c>
+      <c r="G46" t="n">
+        <v>-5.100000000000001</v>
+      </c>
+      <c r="H46" t="n">
+        <v>-5.066666666666666</v>
+      </c>
+      <c r="I46" t="n">
         <v>0.08819171036882004</v>
-      </c>
-      <c r="G46" t="n">
-        <v>5.066666666666663</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="B47" t="n">
-        <v>22.6</v>
+        <v>-22.6</v>
       </c>
       <c r="C47" t="n">
-        <v>22.4</v>
+        <v>-22.4</v>
       </c>
       <c r="D47" t="n">
-        <v>22.3</v>
+        <v>-22.3</v>
       </c>
       <c r="E47" t="n">
-        <v>22.43333333333333</v>
+        <v>-5.100000000000001</v>
       </c>
       <c r="F47" t="n">
+        <v>-4.899999999999999</v>
+      </c>
+      <c r="G47" t="n">
+        <v>-4.800000000000001</v>
+      </c>
+      <c r="H47" t="n">
+        <v>-4.933333333333334</v>
+      </c>
+      <c r="I47" t="n">
         <v>0.08819171036882006</v>
-      </c>
-      <c r="G47" t="n">
-        <v>4.933333333333334</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>19</v>
+        <v>46</v>
       </c>
       <c r="B48" t="n">
-        <v>22.1</v>
+        <v>-22.1</v>
       </c>
       <c r="C48" t="n">
-        <v>22.1</v>
+        <v>-22.1</v>
       </c>
       <c r="D48" t="n">
-        <v>22.4</v>
+        <v>-22.4</v>
       </c>
       <c r="E48" t="n">
-        <v>22.2</v>
+        <v>-4.600000000000001</v>
       </c>
       <c r="F48" t="n">
+        <v>-4.600000000000001</v>
+      </c>
+      <c r="G48" t="n">
+        <v>-4.899999999999999</v>
+      </c>
+      <c r="H48" t="n">
+        <v>-4.7</v>
+      </c>
+      <c r="I48" t="n">
         <v>0.09999999999999906</v>
-      </c>
-      <c r="G48" t="n">
-        <v>4.699999999999999</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>18</v>
+        <v>47</v>
       </c>
       <c r="B49" t="n">
-        <v>22.1</v>
+        <v>-22.1</v>
       </c>
       <c r="C49" t="n">
-        <v>21.9</v>
+        <v>-21.9</v>
       </c>
       <c r="D49" t="n">
-        <v>22</v>
+        <v>-22</v>
       </c>
       <c r="E49" t="n">
-        <v>22</v>
+        <v>-4.600000000000001</v>
       </c>
       <c r="F49" t="n">
+        <v>-4.399999999999999</v>
+      </c>
+      <c r="G49" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="H49" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="I49" t="n">
         <v>0.0577350269189634</v>
-      </c>
-      <c r="G49" t="n">
-        <v>4.5</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>17</v>
+        <v>48</v>
       </c>
       <c r="B50" t="n">
-        <v>21.9</v>
+        <v>-21.9</v>
       </c>
       <c r="C50" t="n">
-        <v>21.7</v>
+        <v>-21.7</v>
       </c>
       <c r="D50" t="n">
-        <v>21.9</v>
+        <v>-21.9</v>
       </c>
       <c r="E50" t="n">
-        <v>21.83333333333333</v>
+        <v>-4.399999999999999</v>
       </c>
       <c r="F50" t="n">
+        <v>-4.199999999999999</v>
+      </c>
+      <c r="G50" t="n">
+        <v>-4.399999999999999</v>
+      </c>
+      <c r="H50" t="n">
+        <v>-4.333333333333332</v>
+      </c>
+      <c r="I50" t="n">
         <v>0.06666666666666643</v>
-      </c>
-      <c r="G50" t="n">
-        <v>4.333333333333332</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>16</v>
+        <v>49</v>
       </c>
       <c r="B51" t="n">
-        <v>20.6</v>
+        <v>-20.6</v>
       </c>
       <c r="C51" t="n">
-        <v>20.5</v>
+        <v>-20.5</v>
       </c>
       <c r="D51" t="n">
-        <v>20.6</v>
+        <v>-20.6</v>
       </c>
       <c r="E51" t="n">
-        <v>20.56666666666667</v>
+        <v>-3.100000000000001</v>
       </c>
       <c r="F51" t="n">
+        <v>-3</v>
+      </c>
+      <c r="G51" t="n">
+        <v>-3.100000000000001</v>
+      </c>
+      <c r="H51" t="n">
+        <v>-3.066666666666668</v>
+      </c>
+      <c r="I51" t="n">
         <v>0.03333333333333381</v>
-      </c>
-      <c r="G51" t="n">
-        <v>3.066666666666666</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="B52" t="n">
-        <v>21.2</v>
+        <v>-21.2</v>
       </c>
       <c r="C52" t="n">
-        <v>21.2</v>
+        <v>-21.2</v>
       </c>
       <c r="D52" t="n">
-        <v>21.3</v>
+        <v>-21.3</v>
       </c>
       <c r="E52" t="n">
-        <v>21.23333333333333</v>
+        <v>-3.699999999999999</v>
       </c>
       <c r="F52" t="n">
-        <v>0.03333333333333381</v>
+        <v>-3.699999999999999</v>
       </c>
       <c r="G52" t="n">
-        <v>3.733333333333334</v>
+        <v>-3.800000000000001</v>
+      </c>
+      <c r="H52" t="n">
+        <v>-3.733333333333333</v>
+      </c>
+      <c r="I52" t="n">
+        <v>0.0333333333333338</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>14</v>
+        <v>51</v>
       </c>
       <c r="B53" t="n">
-        <v>21</v>
+        <v>-21</v>
       </c>
       <c r="C53" t="n">
-        <v>21.3</v>
+        <v>-21.3</v>
       </c>
       <c r="D53" t="n">
-        <v>20.3</v>
+        <v>-20.3</v>
       </c>
       <c r="E53" t="n">
-        <v>20.86666666666666</v>
+        <v>-3.5</v>
       </c>
       <c r="F53" t="n">
-        <v>0.2962731472438529</v>
+        <v>-3.800000000000001</v>
       </c>
       <c r="G53" t="n">
-        <v>3.366666666666664</v>
+        <v>-2.800000000000001</v>
+      </c>
+      <c r="H53" t="n">
+        <v>-3.366666666666667</v>
+      </c>
+      <c r="I53" t="n">
+        <v>0.296273147243853</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>13</v>
+        <v>52</v>
       </c>
       <c r="B54" t="n">
-        <v>21.1</v>
+        <v>-21.1</v>
       </c>
       <c r="C54" t="n">
-        <v>20.9</v>
+        <v>-20.9</v>
       </c>
       <c r="D54" t="n">
-        <v>21</v>
+        <v>-21</v>
       </c>
       <c r="E54" t="n">
-        <v>21</v>
+        <v>-3.600000000000001</v>
       </c>
       <c r="F54" t="n">
+        <v>-3.399999999999999</v>
+      </c>
+      <c r="G54" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="H54" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="I54" t="n">
         <v>0.0577350269189634</v>
-      </c>
-      <c r="G54" t="n">
-        <v>3.5</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>12</v>
+        <v>53</v>
       </c>
       <c r="B55" t="n">
-        <v>20.9</v>
+        <v>-20.9</v>
       </c>
       <c r="C55" t="n">
-        <v>20.8</v>
+        <v>-20.8</v>
       </c>
       <c r="D55" t="n">
-        <v>20.8</v>
+        <v>-20.8</v>
       </c>
       <c r="E55" t="n">
-        <v>20.83333333333333</v>
+        <v>-3.399999999999999</v>
       </c>
       <c r="F55" t="n">
-        <v>0.03333333333333263</v>
+        <v>-3.300000000000001</v>
       </c>
       <c r="G55" t="n">
-        <v>3.333333333333332</v>
+        <v>-3.300000000000001</v>
+      </c>
+      <c r="H55" t="n">
+        <v>-3.333333333333333</v>
+      </c>
+      <c r="I55" t="n">
+        <v>0.03333333333333262</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="B56" t="n">
-        <v>20.6</v>
+        <v>-20.6</v>
       </c>
       <c r="C56" t="n">
-        <v>20.5</v>
+        <v>-20.5</v>
       </c>
       <c r="D56" t="n">
-        <v>20.7</v>
+        <v>-20.7</v>
       </c>
       <c r="E56" t="n">
-        <v>20.6</v>
+        <v>-3.100000000000001</v>
       </c>
       <c r="F56" t="n">
+        <v>-3</v>
+      </c>
+      <c r="G56" t="n">
+        <v>-3.199999999999999</v>
+      </c>
+      <c r="H56" t="n">
+        <v>-3.1</v>
+      </c>
+      <c r="I56" t="n">
         <v>0.05773502691896237</v>
-      </c>
-      <c r="G56" t="n">
-        <v>3.099999999999998</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="B57" t="n">
-        <v>20.5</v>
+        <v>-20.5</v>
       </c>
       <c r="C57" t="n">
-        <v>20.4</v>
+        <v>-20.4</v>
       </c>
       <c r="D57" t="n">
-        <v>20.4</v>
+        <v>-20.4</v>
       </c>
       <c r="E57" t="n">
-        <v>20.43333333333333</v>
+        <v>-3</v>
       </c>
       <c r="F57" t="n">
+        <v>-2.899999999999999</v>
+      </c>
+      <c r="G57" t="n">
+        <v>-2.899999999999999</v>
+      </c>
+      <c r="H57" t="n">
+        <v>-2.933333333333332</v>
+      </c>
+      <c r="I57" t="n">
         <v>0.03333333333333381</v>
-      </c>
-      <c r="G57" t="n">
-        <v>2.933333333333334</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>9</v>
+        <v>56</v>
       </c>
       <c r="B58" t="n">
-        <v>20.4</v>
+        <v>-20.4</v>
       </c>
       <c r="C58" t="n">
-        <v>20.4</v>
+        <v>-20.4</v>
       </c>
       <c r="D58" t="n">
-        <v>20.2</v>
+        <v>-20.2</v>
       </c>
       <c r="E58" t="n">
-        <v>20.33333333333333</v>
+        <v>-2.899999999999999</v>
       </c>
       <c r="F58" t="n">
+        <v>-2.899999999999999</v>
+      </c>
+      <c r="G58" t="n">
+        <v>-2.699999999999999</v>
+      </c>
+      <c r="H58" t="n">
+        <v>-2.833333333333332</v>
+      </c>
+      <c r="I58" t="n">
         <v>0.06666666666666643</v>
-      </c>
-      <c r="G58" t="n">
-        <v>2.833333333333332</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>8</v>
+        <v>57</v>
       </c>
       <c r="B59" t="n">
-        <v>20</v>
+        <v>-20</v>
       </c>
       <c r="C59" t="n">
-        <v>20</v>
+        <v>-20</v>
       </c>
       <c r="D59" t="n">
-        <v>20</v>
+        <v>-20</v>
       </c>
       <c r="E59" t="n">
-        <v>20</v>
+        <v>-2.5</v>
       </c>
       <c r="F59" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="G59" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="H59" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="I59" t="n">
         <v>0</v>
-      </c>
-      <c r="G59" t="n">
-        <v>2.5</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>7</v>
+        <v>58</v>
       </c>
       <c r="B60" t="n">
-        <v>19.9</v>
+        <v>-19.9</v>
       </c>
       <c r="C60" t="n">
-        <v>19.7</v>
+        <v>-19.7</v>
       </c>
       <c r="D60" t="n">
-        <v>19.6</v>
+        <v>-19.6</v>
       </c>
       <c r="E60" t="n">
-        <v>19.73333333333333</v>
+        <v>-2.399999999999999</v>
       </c>
       <c r="F60" t="n">
-        <v>0.08819171036881894</v>
+        <v>-2.199999999999999</v>
       </c>
       <c r="G60" t="n">
-        <v>2.233333333333331</v>
+        <v>-2.100000000000001</v>
+      </c>
+      <c r="H60" t="n">
+        <v>-2.233333333333333</v>
+      </c>
+      <c r="I60" t="n">
+        <v>0.08819171036881893</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>6</v>
+        <v>59</v>
       </c>
       <c r="B61" t="n">
-        <v>19.8</v>
+        <v>-19.8</v>
       </c>
       <c r="C61" t="n">
-        <v>19.6</v>
+        <v>-19.6</v>
       </c>
       <c r="D61" t="n">
-        <v>19.6</v>
+        <v>-19.6</v>
       </c>
       <c r="E61" t="n">
-        <v>19.66666666666667</v>
+        <v>-2.300000000000001</v>
       </c>
       <c r="F61" t="n">
+        <v>-2.100000000000001</v>
+      </c>
+      <c r="G61" t="n">
+        <v>-2.100000000000001</v>
+      </c>
+      <c r="H61" t="n">
+        <v>-2.166666666666668</v>
+      </c>
+      <c r="I61" t="n">
         <v>0.06666666666666643</v>
-      </c>
-      <c r="G61" t="n">
-        <v>2.166666666666668</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>5</v>
+        <v>60</v>
       </c>
       <c r="B62" t="n">
-        <v>19.3</v>
+        <v>-19.3</v>
       </c>
       <c r="C62" t="n">
-        <v>19.2</v>
+        <v>-19.2</v>
       </c>
       <c r="D62" t="n">
-        <v>19.1</v>
+        <v>-19.1</v>
       </c>
       <c r="E62" t="n">
-        <v>19.2</v>
+        <v>-1.800000000000001</v>
       </c>
       <c r="F62" t="n">
+        <v>-1.699999999999999</v>
+      </c>
+      <c r="G62" t="n">
+        <v>-1.600000000000001</v>
+      </c>
+      <c r="H62" t="n">
+        <v>-1.7</v>
+      </c>
+      <c r="I62" t="n">
         <v>0.05773502691896237</v>
-      </c>
-      <c r="G62" t="n">
-        <v>1.699999999999999</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>4</v>
+        <v>61</v>
       </c>
       <c r="B63" t="n">
-        <v>19.4</v>
+        <v>-19.4</v>
       </c>
       <c r="C63" t="n">
-        <v>19.2</v>
+        <v>-19.2</v>
       </c>
       <c r="D63" t="n">
-        <v>19.2</v>
+        <v>-19.2</v>
       </c>
       <c r="E63" t="n">
-        <v>19.26666666666667</v>
+        <v>-1.899999999999999</v>
       </c>
       <c r="F63" t="n">
+        <v>-1.699999999999999</v>
+      </c>
+      <c r="G63" t="n">
+        <v>-1.699999999999999</v>
+      </c>
+      <c r="H63" t="n">
+        <v>-1.766666666666666</v>
+      </c>
+      <c r="I63" t="n">
         <v>0.06666666666666643</v>
-      </c>
-      <c r="G63" t="n">
-        <v>1.766666666666666</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>3</v>
+        <v>62</v>
       </c>
       <c r="B64" t="n">
-        <v>18.4</v>
+        <v>-18.4</v>
       </c>
       <c r="C64" t="n">
-        <v>18.3</v>
+        <v>-18.3</v>
       </c>
       <c r="D64" t="n">
-        <v>18.6</v>
+        <v>-18.6</v>
       </c>
       <c r="E64" t="n">
-        <v>18.43333333333333</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="F64" t="n">
+        <v>-0.8000000000000007</v>
+      </c>
+      <c r="G64" t="n">
+        <v>-1.100000000000001</v>
+      </c>
+      <c r="H64" t="n">
+        <v>-0.9333333333333336</v>
+      </c>
+      <c r="I64" t="n">
         <v>0.08819171036882006</v>
-      </c>
-      <c r="G64" t="n">
-        <v>0.9333333333333336</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>2</v>
+        <v>63</v>
       </c>
       <c r="B65" t="n">
-        <v>18.2</v>
+        <v>-18.2</v>
       </c>
       <c r="C65" t="n">
-        <v>18.1</v>
+        <v>-18.1</v>
       </c>
       <c r="D65" t="n">
-        <v>17.9</v>
+        <v>-17.9</v>
       </c>
       <c r="E65" t="n">
-        <v>18.06666666666667</v>
+        <v>-0.6999999999999993</v>
       </c>
       <c r="F65" t="n">
+        <v>-0.6000000000000014</v>
+      </c>
+      <c r="G65" t="n">
+        <v>-0.3999999999999986</v>
+      </c>
+      <c r="H65" t="n">
+        <v>-0.5666666666666664</v>
+      </c>
+      <c r="I65" t="n">
         <v>0.08819171036882006</v>
-      </c>
-      <c r="G65" t="n">
-        <v>0.5666666666666664</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>1</v>
+        <v>64</v>
       </c>
       <c r="B66" t="n">
-        <v>18.1</v>
+        <v>-18.1</v>
       </c>
       <c r="C66" t="n">
-        <v>18</v>
+        <v>-18</v>
       </c>
       <c r="D66" t="n">
-        <v>18.3</v>
+        <v>-18.3</v>
       </c>
       <c r="E66" t="n">
-        <v>18.13333333333334</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="F66" t="n">
-        <v>0.08819171036881983</v>
+        <v>-0.5</v>
       </c>
       <c r="G66" t="n">
-        <v>0.6333333333333364</v>
+        <v>-0.8000000000000007</v>
+      </c>
+      <c r="H66" t="n">
+        <v>-0.6333333333333341</v>
+      </c>
+      <c r="I66" t="n">
+        <v>0.08819171036881981</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="B67" t="n">
-        <v>17.6</v>
+        <v>-17.6</v>
       </c>
       <c r="C67" t="n">
-        <v>17.4</v>
+        <v>-17.4</v>
       </c>
       <c r="D67" t="n">
-        <v>17.5</v>
+        <v>-17.5</v>
       </c>
       <c r="E67" t="n">
-        <v>17.5</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="F67" t="n">
-        <v>0.0577350269189634</v>
+        <v>0.1000000000000014</v>
       </c>
       <c r="G67" t="n">
         <v>0</v>
+      </c>
+      <c r="H67" t="n">
+        <v>0</v>
+      </c>
+      <c r="I67" t="n">
+        <v>0.0577350269189634</v>
       </c>
     </row>
   </sheetData>

</xml_diff>